<commit_message>
Bundle the asymmetry data for the hepgen branch
asymmetries_for_hepgen.tar.gz: the four sets as published, a README stating what
each one is and how to turn a model into it, and load_asymmetries.py which does
that in one call.  Nothing in the bundle converts the data -- the model is
converted instead, because every pre-applied conversion we inherited turned out
to be wrong: CLAS12 by a factor four, Hall-A 2011 by gamma, and the two CLAS6
digitisations by 1.5 and 1.3 in their errors.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pi0_eta_database.xlsx
+++ b/pi0_eta_database.xlsx
@@ -1099,7 +1099,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Zhao et al., PLB 789 426 (2019), figure extraction</t>
+          <t>Zhao et al., PLB 789 426 (2019), figure 5 read from the vector PDF</t>
         </is>
       </c>
     </row>
@@ -54580,13 +54580,13 @@
         <v>-0.26</v>
       </c>
       <c r="H64" s="6" t="n">
-        <v>0.2122</v>
+        <v>0.212</v>
       </c>
       <c r="I64" s="6" t="n">
-        <v>0.027</v>
+        <v>0.035</v>
       </c>
       <c r="J64" s="6" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.0478</v>
       </c>
       <c r="K64" t="n">
         <v>5.776</v>
@@ -54598,7 +54598,7 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>Zhao et al., PLB 789 426 (2019), figure extraction</t>
+          <t>Zhao et al., PLB 789 426 (2019), figure 5 read from the vector PDF</t>
         </is>
       </c>
     </row>
@@ -54636,10 +54636,10 @@
         <v>0.0951</v>
       </c>
       <c r="I65" s="6" t="n">
-        <v>0.026</v>
+        <v>0.034</v>
       </c>
       <c r="J65" s="6" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.0243</v>
       </c>
       <c r="K65" t="n">
         <v>5.776</v>
@@ -54651,7 +54651,7 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>Zhao et al., PLB 789 426 (2019), figure extraction</t>
+          <t>Zhao et al., PLB 789 426 (2019), figure 5 read from the vector PDF</t>
         </is>
       </c>
     </row>
@@ -54689,10 +54689,10 @@
         <v>0.1231</v>
       </c>
       <c r="I66" s="6" t="n">
-        <v>0.029</v>
+        <v>0.037</v>
       </c>
       <c r="J66" s="6" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.0393</v>
       </c>
       <c r="K66" t="n">
         <v>5.776</v>
@@ -54704,7 +54704,7 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>Zhao et al., PLB 789 426 (2019), figure extraction</t>
+          <t>Zhao et al., PLB 789 426 (2019), figure 5 read from the vector PDF</t>
         </is>
       </c>
     </row>
@@ -54739,13 +54739,13 @@
         <v>-0.258</v>
       </c>
       <c r="H67" s="6" t="n">
-        <v>0.1471</v>
+        <v>0.147</v>
       </c>
       <c r="I67" s="6" t="n">
-        <v>0.032</v>
+        <v>0.04</v>
       </c>
       <c r="J67" s="6" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.0346</v>
       </c>
       <c r="K67" t="n">
         <v>5.776</v>
@@ -54757,7 +54757,7 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>Zhao et al., PLB 789 426 (2019), figure extraction</t>
+          <t>Zhao et al., PLB 789 426 (2019), figure 5 read from the vector PDF</t>
         </is>
       </c>
     </row>
@@ -54792,13 +54792,13 @@
         <v>-0.577</v>
       </c>
       <c r="H68" s="6" t="n">
-        <v>0.1331</v>
+        <v>0.133</v>
       </c>
       <c r="I68" s="6" t="n">
-        <v>0.026</v>
+        <v>0.034</v>
       </c>
       <c r="J68" s="6" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.0218</v>
       </c>
       <c r="K68" t="n">
         <v>5.776</v>
@@ -54810,7 +54810,7 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>Zhao et al., PLB 789 426 (2019), figure extraction</t>
+          <t>Zhao et al., PLB 789 426 (2019), figure 5 read from the vector PDF</t>
         </is>
       </c>
     </row>
@@ -54845,13 +54845,13 @@
         <v>-1.13</v>
       </c>
       <c r="H69" s="6" t="n">
-        <v>0.1631</v>
+        <v>0.163</v>
       </c>
       <c r="I69" s="6" t="n">
-        <v>0.035</v>
+        <v>0.043</v>
       </c>
       <c r="J69" s="6" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.0367</v>
       </c>
       <c r="K69" t="n">
         <v>5.776</v>
@@ -54863,7 +54863,7 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>Zhao et al., PLB 789 426 (2019), figure extraction</t>
+          <t>Zhao et al., PLB 789 426 (2019), figure 5 read from the vector PDF</t>
         </is>
       </c>
     </row>
@@ -54898,13 +54898,13 @@
         <v>-0.318</v>
       </c>
       <c r="H70" s="6" t="n">
-        <v>0.2031</v>
+        <v>0.2081</v>
       </c>
       <c r="I70" s="6" t="n">
-        <v>0.0528</v>
+        <v>0.0597</v>
       </c>
       <c r="J70" s="6" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.0641</v>
       </c>
       <c r="K70" t="n">
         <v>5.776</v>
@@ -54916,7 +54916,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>Zhao et al., PLB 789 426 (2019), figure extraction</t>
+          <t>Zhao et al., PLB 789 426 (2019), figure 5 read from the vector PDF</t>
         </is>
       </c>
     </row>
@@ -54951,13 +54951,13 @@
         <v>-0.593</v>
       </c>
       <c r="H71" s="6" t="n">
-        <v>0.131</v>
+        <v>0.1377</v>
       </c>
       <c r="I71" s="6" t="n">
-        <v>0.0238</v>
+        <v>0.0313</v>
       </c>
       <c r="J71" s="6" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.0366</v>
       </c>
       <c r="K71" t="n">
         <v>5.776</v>
@@ -54969,7 +54969,7 @@
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>Zhao et al., PLB 789 426 (2019), figure extraction</t>
+          <t>Zhao et al., PLB 789 426 (2019), figure 5 read from the vector PDF</t>
         </is>
       </c>
     </row>
@@ -55004,13 +55004,13 @@
         <v>-1.19</v>
       </c>
       <c r="H72" s="6" t="n">
-        <v>0.137</v>
+        <v>0.1436</v>
       </c>
       <c r="I72" s="6" t="n">
-        <v>0.0218</v>
+        <v>0.0293</v>
       </c>
       <c r="J72" s="6" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.0395</v>
       </c>
       <c r="K72" t="n">
         <v>5.776</v>
@@ -55022,7 +55022,7 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>Zhao et al., PLB 789 426 (2019), figure extraction</t>
+          <t>Zhao et al., PLB 789 426 (2019), figure 5 read from the vector PDF</t>
         </is>
       </c>
     </row>
@@ -55057,13 +55057,13 @@
         <v>-0.318</v>
       </c>
       <c r="H73" s="6" t="n">
-        <v>0.1891</v>
+        <v>0.1944</v>
       </c>
       <c r="I73" s="6" t="n">
-        <v>0.0668</v>
+        <v>0.0733</v>
       </c>
       <c r="J73" s="6" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.0447</v>
       </c>
       <c r="K73" t="n">
         <v>5.776</v>
@@ -55075,7 +55075,7 @@
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>Zhao et al., PLB 789 426 (2019), figure extraction</t>
+          <t>Zhao et al., PLB 789 426 (2019), figure 5 read from the vector PDF</t>
         </is>
       </c>
     </row>
@@ -55110,13 +55110,13 @@
         <v>-0.601</v>
       </c>
       <c r="H74" s="6" t="n">
-        <v>0.1771</v>
+        <v>0.1827</v>
       </c>
       <c r="I74" s="6" t="n">
-        <v>0.0308</v>
+        <v>0.0381</v>
       </c>
       <c r="J74" s="6" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.0437</v>
       </c>
       <c r="K74" t="n">
         <v>5.776</v>
@@ -55128,7 +55128,7 @@
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>Zhao et al., PLB 789 426 (2019), figure extraction</t>
+          <t>Zhao et al., PLB 789 426 (2019), figure 5 read from the vector PDF</t>
         </is>
       </c>
     </row>
@@ -55163,13 +55163,13 @@
         <v>-1.21</v>
       </c>
       <c r="H75" s="6" t="n">
-        <v>0.1991</v>
+        <v>0.2042</v>
       </c>
       <c r="I75" s="6" t="n">
-        <v>0.0238</v>
+        <v>0.0313</v>
       </c>
       <c r="J75" s="6" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.0438</v>
       </c>
       <c r="K75" t="n">
         <v>5.776</v>
@@ -55181,7 +55181,7 @@
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>Zhao et al., PLB 789 426 (2019), figure extraction</t>
+          <t>Zhao et al., PLB 789 426 (2019), figure 5 read from the vector PDF</t>
         </is>
       </c>
     </row>

</xml_diff>